<commit_message>
Fixed bugs related to tracking and rendering of VOBI (victim of back invalidation).
</commit_message>
<xml_diff>
--- a/test/tcs01_FIFO/golden_output.xlsx
+++ b/test/tcs01_FIFO/golden_output.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,12 @@
       <i val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -98,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -135,6 +141,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -505,16 +514,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.78" customWidth="1" min="1" max="1"/>
-    <col width="27.78" customWidth="1" min="2" max="2"/>
-    <col width="27.78" customWidth="1" min="3" max="3"/>
-    <col width="27.78" customWidth="1" min="4" max="4"/>
-    <col width="27.78" customWidth="1" min="5" max="5"/>
-    <col width="27.78" customWidth="1" min="6" max="6"/>
-    <col width="27.78" customWidth="1" min="7" max="7"/>
+    <col width="34.78" customWidth="1" min="2" max="2"/>
+    <col width="34.78" customWidth="1" min="3" max="3"/>
+    <col width="34.78" customWidth="1" min="4" max="4"/>
+    <col width="34.78" customWidth="1" min="5" max="5"/>
+    <col width="34.78" customWidth="1" min="6" max="6"/>
+    <col width="34.78" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28.8" customHeight="1">
@@ -561,37 +570,37 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>20,200
-(V:T, D:T, MCA:T, TS:0, LAT:0)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
           <t>20,-99999
-(V:T, D:F, MCA:T, TS:0, LAT:0)</t>
+(V:T, D:F, VOBI:F, MCA:T, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
     </row>
@@ -602,37 +611,37 @@
       <c r="B3" s="6" t="inlineStr">
         <is>
           <t>20,200
-(V:T, D:T, MCA:F, TS:0, LAT:0)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>21,300
-(V:T, D:T, MCA:T, TS:1, LAT:1)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:1, LAT:1)</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
           <t>20,-99999
-(V:T, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
           <t>21,-99999
-(V:T, D:F, MCA:T, TS:1, LAT:1)</t>
+(V:T, D:F, VOBI:F, MCA:T, TS:1, LAT:1)</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
     </row>
@@ -643,37 +652,37 @@
       <c r="B4" s="6" t="inlineStr">
         <is>
           <t>20,200
-(V:T, D:T, MCA:F, TS:0, LAT:2)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:0, LAT:2)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
           <t>21,300
-(V:T, D:T, MCA:F, TS:1, LAT:1)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>20,-99999
-(V:T, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
           <t>21,-99999
-(V:T, D:F, MCA:F, TS:1, LAT:1)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
     </row>
@@ -684,37 +693,37 @@
       <c r="B5" s="6" t="inlineStr">
         <is>
           <t>20,200
-(V:T, D:T, MCA:F, TS:0, LAT:3)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:0, LAT:3)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
           <t>21,300
-(V:T, D:T, MCA:F, TS:1, LAT:1)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>20,-99999
-(V:T, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
           <t>21,-99999
-(V:T, D:F, MCA:F, TS:1, LAT:1)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
     </row>
@@ -725,37 +734,37 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:T, MCA:T, TS:4, LAT:4)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:4, LAT:4)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
           <t>21,300
-(V:T, D:T, MCA:F, TS:1, LAT:1)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>20,200
-(V:T, D:T, MCA:T, TS:3, LAT:3)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:3, LAT:3)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
           <t>21,-99999
-(V:T, D:F, MCA:F, TS:1, LAT:1)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
           <t>22,-99999
-(V:T, D:F, MCA:T, TS:2, LAT:2)</t>
+(V:T, D:F, VOBI:F, MCA:T, TS:2, LAT:2)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
           <t>0,0
-(V:F, D:F, MCA:F, TS:0, LAT:0)</t>
+(V:F, D:F, VOBI:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
     </row>
@@ -766,37 +775,37 @@
       <c r="B7" s="6" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:T, MCA:F, TS:4, LAT:4)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:4, LAT:4)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:T, MCA:T, TS:5, LAT:5)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:5, LAT:5)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
           <t>20,200
-(V:T, D:T, MCA:F, TS:3, LAT:3)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:3, LAT:3)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>21,300
-(V:T, D:T, MCA:T, TS:5, LAT:5)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:5, LAT:5)</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
           <t>22,-99999
-(V:T, D:F, MCA:F, TS:2, LAT:2)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:2, LAT:2)</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
           <t>23,-99999
-(V:T, D:F, MCA:T, TS:4, LAT:4)</t>
+(V:T, D:F, VOBI:F, MCA:T, TS:4, LAT:4)</t>
         </is>
       </c>
     </row>
@@ -807,37 +816,37 @@
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>20,201
-(V:T, D:T, MCA:T, TS:6, LAT:6)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:6, LAT:6)</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:T, MCA:F, TS:5, LAT:5)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:5, LAT:5)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
           <t>20,200
-(V:T, D:T, MCA:F, TS:3, LAT:6)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:3, LAT:6)</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>21,300
-(V:T, D:T, MCA:F, TS:5, LAT:5)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:5, LAT:5)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:T, MCA:T, TS:7, LAT:7)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:7, LAT:7)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>23,-99999
-(V:T, D:F, MCA:F, TS:4, LAT:4)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:4, LAT:4)</t>
         </is>
       </c>
     </row>
@@ -848,37 +857,37 @@
       <c r="B9" s="6" t="inlineStr">
         <is>
           <t>20,201
-(V:T, D:T, MCA:F, TS:6, LAT:6)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:6, LAT:6)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
           <t>21,301
-(V:T, D:T, MCA:T, TS:7, LAT:7)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:7, LAT:7)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
           <t>20,200
-(V:T, D:T, MCA:F, TS:3, LAT:6)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:3, LAT:6)</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
           <t>21,300
-(V:T, D:T, MCA:F, TS:5, LAT:8)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:5, LAT:8)</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:T, MCA:F, TS:7, LAT:7)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:7, LAT:7)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:T, MCA:T, TS:9, LAT:9)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:9, LAT:9)</t>
         </is>
       </c>
     </row>
@@ -889,37 +898,37 @@
       <c r="B10" s="5" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:F, MCA:T, TS:8, LAT:8)</t>
+(V:T, D:F, VOBI:F, MCA:T, TS:8, LAT:8)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
           <t>21,301
-(V:T, D:T, MCA:F, TS:7, LAT:7)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:7, LAT:7)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
           <t>20,201
-(V:T, D:T, MCA:T, TS:11, LAT:11)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:11, LAT:11)</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
           <t>21,300
-(V:T, D:T, MCA:F, TS:5, LAT:8)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:5, LAT:8)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:T, MCA:F, TS:7, LAT:10)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:7, LAT:10)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:T, MCA:F, TS:9, LAT:9)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:9, LAT:9)</t>
         </is>
       </c>
     </row>
@@ -930,37 +939,37 @@
       <c r="B11" s="7" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:F, MCA:F, TS:8, LAT:8)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:8, LAT:8)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:F, MCA:T, TS:9, LAT:9)</t>
+(V:T, D:F, VOBI:F, MCA:T, TS:9, LAT:9)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
           <t>20,201
-(V:T, D:T, MCA:F, TS:11, LAT:11)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:11, LAT:11)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
           <t>21,301
-(V:T, D:T, MCA:T, TS:13, LAT:13)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:13, LAT:13)</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:T, MCA:F, TS:7, LAT:10)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:7, LAT:10)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:T, MCA:F, TS:9, LAT:12)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:9, LAT:12)</t>
         </is>
       </c>
     </row>
@@ -971,37 +980,37 @@
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>22,401
-(V:T, D:T, MCA:T, TS:10, LAT:10)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:10, LAT:10)</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:F, MCA:F, TS:9, LAT:9)</t>
+(V:T, D:F, VOBI:F, MCA:F, TS:9, LAT:9)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
           <t>20,201
-(V:T, D:T, MCA:F, TS:11, LAT:11)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:11, LAT:11)</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
           <t>21,301
-(V:T, D:T, MCA:F, TS:13, LAT:13)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:13, LAT:13)</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:T, MCA:F, TS:7, LAT:10)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:7, LAT:10)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:T, MCA:F, TS:9, LAT:12)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:9, LAT:12)</t>
         </is>
       </c>
     </row>
@@ -1012,37 +1021,37 @@
       <c r="B13" s="6" t="inlineStr">
         <is>
           <t>22,401
-(V:T, D:T, MCA:F, TS:10, LAT:10)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:10, LAT:10)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
           <t>23,501
-(V:T, D:T, MCA:T, TS:11, LAT:11)</t>
+(V:T, D:T, VOBI:F, MCA:T, TS:11, LAT:11)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
           <t>20,201
-(V:T, D:T, MCA:F, TS:11, LAT:11)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:11, LAT:11)</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
           <t>21,301
-(V:T, D:T, MCA:F, TS:13, LAT:13)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:13, LAT:13)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
           <t>22,400
-(V:T, D:T, MCA:F, TS:7, LAT:10)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:7, LAT:10)</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
           <t>23,500
-(V:T, D:T, MCA:F, TS:9, LAT:12)</t>
+(V:T, D:T, VOBI:F, MCA:F, TS:9, LAT:12)</t>
         </is>
       </c>
     </row>
@@ -1108,6 +1117,18 @@
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Victim Of Back Invalidation (VOBI:T), possibly subsequently populated with valid data</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Sample</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Unused entry available for use (V:F)</t>
         </is>

</xml_diff>